<commit_message>
Fix reduction determinism (sorted cand + PYTHONHASHSEED=0), switch E3 figure x-axis to max_total, relaunch E3 sweep
</commit_message>
<xml_diff>
--- a/figures/图表.xlsx
+++ b/figures/图表.xlsx
@@ -9,8 +9,9 @@
   <sheets>
     <sheet name="E1_encoding_matrix" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="E1_alert" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="E2_slot_equivalence" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="StreamSpot" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="E3_strength_sweep" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="E2_slot_equivalence" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="StreamSpot" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -510,6 +511,188 @@
 </chartSpace>
 </file>
 
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Detection quality vs reduction budget</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'E3_strength_sweep'!B1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'E3_strength_sweep'!$A$2:$A$5</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'E3_strength_sweep'!$B$2:$B$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'E3_strength_sweep'!C1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'E3_strength_sweep'!$A$2:$A$5</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'E3_strength_sweep'!$C$2:$C$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="2"/>
+          <order val="2"/>
+          <tx>
+            <strRef>
+              <f>'E3_strength_sweep'!D1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'E3_strength_sweep'!$A$2:$A$5</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'E3_strength_sweep'!$D$2:$D$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>max_total (template instance budget)</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>node best-F1</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
@@ -547,6 +730,33 @@
       <rowOff>0</rowOff>
     </from>
     <ext cx="5760000" cy="3240000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>7</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6480000" cy="3600000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>
@@ -1051,6 +1261,141 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:F5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>max_total</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>dual_naive</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>rate</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>nodes_kept</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>edge_cut</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>250</v>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>0.1356</v>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>0.008274999999999999</v>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>0.135775</v>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>0.9713179397753898</v>
+      </c>
+      <c r="F2" s="2" t="n">
+        <v>0.119151128637896</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>1000</v>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>0.138625</v>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>0.00805</v>
+      </c>
+      <c r="D3" s="2" t="n">
+        <v>0.13885</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>0.937594786681343</v>
+      </c>
+      <c r="F3" s="2" t="n">
+        <v>0.165719308732626</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>4000</v>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>0.11735</v>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>0.0063</v>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>0.117525</v>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>0.9356970487343051</v>
+      </c>
+      <c r="F4" s="2" t="n">
+        <v>0.2605733566577428</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>16000</v>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>0.1197</v>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>0.008225</v>
+      </c>
+      <c r="D5" s="2" t="n">
+        <v>0.1199333333333333</v>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>0.922217229087544</v>
+      </c>
+      <c r="F5" s="2" t="n">
+        <v>0.170398105559511</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1180,7 +1525,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
E3 strength sweep: fig2 + Excel rebuild, full-scale sweep queued
- results/e3_strength_sweep_all.csv: fresh small-window sweep (3 truncated
  windows x 4 max_total budgets x 3 encodings), replaces the internally
  inconsistent 09-16 pull; edge-reduction ratios span 12.3-46.4%
- make_fig_png.py: panel (a) = five-level encoding spectrum incl. semantic-only
  (dual annotation); panel (b) = node best-F1 vs REALIZED edge-reduction ratio,
  one curve per window, production-setting (15%) reference line. x=0 identity
  anchors deliberately NOT joined (reduced-unit positives not comparable)
- make_excel.py: header-row filter, e1b/ and e3full/ staging dirs; 图表.xlsx
  regenerated (5 sheets incl. StreamSpot)
- run_e3_full.sh + e3full_queue.sh: full-scale sweep drivers (4 large
  partitions x 4 budgets, wave-parallel, training-reduction caches warm)
</commit_message>
<xml_diff>
--- a/figures/图表.xlsx
+++ b/figures/图表.xlsx
@@ -261,6 +261,30 @@
             </numRef>
           </val>
         </ser>
+        <ser>
+          <idx val="4"/>
+          <order val="4"/>
+          <tx>
+            <strRef>
+              <f>'E1_encoding_matrix'!F1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'E1_encoding_matrix'!$A$2:$A$3</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'E1_encoding_matrix'!$F$2:$F$3</f>
+            </numRef>
+          </val>
+        </ser>
         <gapWidth val="150"/>
         <axId val="10"/>
         <axId val="100"/>
@@ -442,6 +466,30 @@
           <val>
             <numRef>
               <f>'E1_alert'!$E$2:$E$3</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="4"/>
+          <order val="4"/>
+          <tx>
+            <strRef>
+              <f>'E1_alert'!F1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'E1_alert'!$A$2:$A$3</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'E1_alert'!$F$2:$F$3</f>
             </numRef>
           </val>
         </ser>
@@ -1063,7 +1111,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
@@ -1071,7 +1119,8 @@
     <col width="11" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1102,6 +1151,11 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
+          <t>semantic_only</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t>MEAN</t>
         </is>
       </c>
@@ -1125,7 +1179,10 @@
         <v>0.1232428571428571</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>0.09413571428571428</v>
+        <v>0.0008</v>
+      </c>
+      <c r="G2" s="2" t="n">
+        <v>0.07546857142857143</v>
       </c>
     </row>
     <row r="3">
@@ -1147,7 +1204,10 @@
         <v>0.09244285714285715</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>0.1094928571428571</v>
+        <v>0.003271428571428571</v>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>0.08824857142857143</v>
       </c>
     </row>
   </sheetData>
@@ -1162,7 +1222,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
@@ -1170,7 +1230,8 @@
     <col width="11" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1201,6 +1262,11 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
+          <t>semantic_only</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t>MEAN</t>
         </is>
       </c>
@@ -1224,7 +1290,10 @@
         <v>0.5785857142857144</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>0.4442571428571429</v>
+        <v>0.0119</v>
+      </c>
+      <c r="G2" s="2" t="n">
+        <v>0.3577857142857143</v>
       </c>
     </row>
     <row r="3">
@@ -1246,7 +1315,10 @@
         <v>0.6977714285714286</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>0.528675</v>
+        <v>0.05832857142857143</v>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>0.4346057142857143</v>
       </c>
     </row>
   </sheetData>
@@ -1309,19 +1381,19 @@
         <v>250</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>0.1356</v>
+        <v>0.08296666666666667</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>0.008274999999999999</v>
+        <v>0.008033333333333333</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>0.135775</v>
+        <v>0.08323333333333334</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>0.9713179397753898</v>
+        <v>0.9634389940406055</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>0.119151128637896</v>
+        <v>0.2430422737314475</v>
       </c>
     </row>
     <row r="3">
@@ -1329,19 +1401,19 @@
         <v>1000</v>
       </c>
       <c r="B3" s="2" t="n">
-        <v>0.138625</v>
+        <v>0.08256666666666666</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>0.00805</v>
+        <v>0.008333333333333333</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>0.13885</v>
+        <v>0.08276666666666667</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>0.937594786681343</v>
+        <v>0.9176986324944303</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>0.165719308732626</v>
+        <v>0.2589864300001248</v>
       </c>
     </row>
     <row r="4">
@@ -1349,19 +1421,19 @@
         <v>4000</v>
       </c>
       <c r="B4" s="2" t="n">
-        <v>0.11735</v>
+        <v>0.09100000000000001</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>0.0063</v>
+        <v>0.009066666666666667</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>0.117525</v>
+        <v>0.09116666666666667</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>0.9356970487343051</v>
+        <v>0.9088687905344656</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>0.2605733566577428</v>
+        <v>0.275563071918449</v>
       </c>
     </row>
     <row r="5">
@@ -1369,19 +1441,19 @@
         <v>16000</v>
       </c>
       <c r="B5" s="2" t="n">
-        <v>0.1197</v>
+        <v>0.09100000000000001</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>0.008225</v>
+        <v>0.009066666666666667</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>0.1199333333333333</v>
+        <v>0.09116666666666667</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>0.922217229087544</v>
+        <v>0.9088687905344656</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>0.170398105559511</v>
+        <v>0.275563071918449</v>
       </c>
     </row>
   </sheetData>

</xml_diff>